<commit_message>
Redesign table structure and improve styling - Replace CSS Grid with HTML table for better column alignment - Remove header icons for cleaner appearance - Center all table headers - Fix data display issues with proper table structure
</commit_message>
<xml_diff>
--- a/public/Vessels Log.xlsx
+++ b/public/Vessels Log.xlsx
@@ -8359,7 +8359,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H88"/>
+  <dimension ref="A1:H89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15.85546875" customWidth="1" min="1" max="1"/>
@@ -10911,7 +10911,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>test1</t>
+          <t>test12</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -10947,26 +10947,26 @@
     </row>
     <row r="86">
       <c r="A86" t="n">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>test2</t>
+          <t>testing21</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>UNMOORING</t>
+          <t>SHIFTING</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>test2</t>
+          <t>testing2</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>test2</t>
+          <t>testing2</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
@@ -10987,31 +10987,31 @@
     </row>
     <row r="87">
       <c r="A87" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>testing2</t>
+          <t>testing12</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>SHIFTING</t>
+          <t>W/ MOORING BUOY</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>testing2</t>
+          <t>testing1</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>testing2</t>
+          <t>testing1</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>2025-10-30</t>
+          <t>2025-10-29</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
@@ -11021,17 +11021,17 @@
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>Foreign</t>
+          <t>Local</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="n">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>testing1</t>
+          <t>tset1</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -11041,25 +11041,65 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>testing1</t>
+          <t>tset</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>testing1</t>
+          <t>tset</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>2025-10-29</t>
+          <t>2025-10-31</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>08:02</t>
+          <t>10:31</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="n">
+        <v>88</v>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>test21</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>W/ MOORING BUOY</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>test2</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>test2</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>2025-10-30</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>10:36</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
         <is>
           <t>Local</t>
         </is>

</xml_diff>

<commit_message>
Add Time Finished field to scheduling and reports, improve weather API integration, fix calendar display, and enhance vessel editing
</commit_message>
<xml_diff>
--- a/public/Vessels Log.xlsx
+++ b/public/Vessels Log.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -57,12 +57,6 @@
       <b val="1"/>
       <color indexed="8"/>
       <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <sz val="8"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -400,7 +394,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="30">
+  <dxfs count="33">
     <dxf>
       <font>
         <name val="Calibri"/>
@@ -426,33 +420,8 @@
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <condense val="0"/>
-        <color theme="1"/>
-        <extend val="0"/>
-        <sz val="10"/>
-        <vertAlign val="baseline"/>
-      </font>
-      <alignment horizontal="center" vertical="center"/>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right/>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
+        <vertical/>
+        <horizontal/>
       </border>
     </dxf>
     <dxf>
@@ -492,12 +461,12 @@
         <outline val="0"/>
         <shadow val="0"/>
         <condense val="0"/>
-        <color indexed="8"/>
+        <color theme="1"/>
         <extend val="0"/>
         <sz val="10"/>
         <vertAlign val="baseline"/>
       </font>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
       <border>
         <left style="thin">
           <color indexed="64"/>
@@ -828,6 +797,64 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <border>
         <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <condense val="0"/>
+        <color indexed="8"/>
+        <extend val="0"/>
+        <sz val="10"/>
+        <vertAlign val="baseline"/>
+      </font>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <condense val="0"/>
+        <color indexed="8"/>
+        <extend val="0"/>
+        <sz val="10"/>
+        <vertAlign val="baseline"/>
+      </font>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <border>
+        <left style="thin">
           <color auto="1"/>
         </left>
         <right style="thin">
@@ -1005,6 +1032,60 @@
         </right>
         <top/>
         <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <condense val="0"/>
+        <color theme="1"/>
+        <extend val="0"/>
+        <sz val="10"/>
+        <vertAlign val="baseline"/>
+      </font>
+      <alignment horizontal="center" vertical="center"/>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <condense val="0"/>
+        <color theme="1"/>
+        <extend val="0"/>
+        <sz val="10"/>
+        <vertAlign val="baseline"/>
+      </font>
+      <alignment horizontal="center" vertical="center"/>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
       </border>
     </dxf>
     <dxf>
@@ -1271,51 +1352,54 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table3" displayName="Table3" ref="A1:H74" headerRowCount="1" totalsRowShown="0" headerRowDxfId="29" tableBorderDxfId="28">
-  <autoFilter ref="A1:H74"/>
-  <tableColumns count="8">
-    <tableColumn id="1" name="No." dataDxfId="27"/>
-    <tableColumn id="2" name="Vessel" dataDxfId="26"/>
-    <tableColumn id="8" name="Service" dataDxfId="25"/>
-    <tableColumn id="3" name="Control Number" dataDxfId="24"/>
-    <tableColumn id="4" name="Voyage Number" dataDxfId="23"/>
-    <tableColumn id="5" name="Date" dataDxfId="22"/>
-    <tableColumn id="6" name="Time" dataDxfId="1"/>
-    <tableColumn id="7" name="Vessel Type" dataDxfId="0"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table3" displayName="Table3" ref="A1:I74" headerRowCount="1" totalsRowShown="0" headerRowDxfId="32" tableBorderDxfId="31">
+  <autoFilter ref="A1:I74"/>
+  <tableColumns count="9">
+    <tableColumn id="1" name="No." dataDxfId="30"/>
+    <tableColumn id="2" name="Vessel" dataDxfId="29"/>
+    <tableColumn id="8" name="Service" dataDxfId="28"/>
+    <tableColumn id="3" name="Control Number" dataDxfId="27"/>
+    <tableColumn id="4" name="Voyage Number" dataDxfId="26"/>
+    <tableColumn id="5" name="Date" dataDxfId="25"/>
+    <tableColumn id="6" name="Time" dataDxfId="24"/>
+    <tableColumn id="9" name="Time Finished" dataDxfId="0"/>
+    <tableColumn id="7" name="Vessel Type" dataDxfId="23"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Table2" displayName="Table2" ref="A1:H148" headerRowCount="1" totalsRowShown="0" headerRowDxfId="21" tableBorderDxfId="20">
-  <autoFilter ref="A1:H148"/>
-  <tableColumns count="8">
-    <tableColumn id="1" name="No." dataDxfId="19"/>
-    <tableColumn id="2" name="Vessel" dataDxfId="18"/>
-    <tableColumn id="3" name="Service" dataDxfId="17"/>
-    <tableColumn id="4" name="Control Number" dataDxfId="16"/>
-    <tableColumn id="5" name="Voyage Number" dataDxfId="15"/>
-    <tableColumn id="6" name="Date" dataDxfId="14"/>
-    <tableColumn id="7" name="Time" dataDxfId="3"/>
-    <tableColumn id="8" name="Vessel Type" dataDxfId="2"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Table2" displayName="Table2" ref="A1:I148" headerRowCount="1" totalsRowShown="0" headerRowDxfId="22" tableBorderDxfId="21">
+  <autoFilter ref="A1:I148"/>
+  <tableColumns count="9">
+    <tableColumn id="1" name="No." dataDxfId="20"/>
+    <tableColumn id="2" name="Vessel" dataDxfId="19"/>
+    <tableColumn id="3" name="Service" dataDxfId="18"/>
+    <tableColumn id="4" name="Control Number" dataDxfId="17"/>
+    <tableColumn id="5" name="Voyage Number" dataDxfId="16"/>
+    <tableColumn id="6" name="Date" dataDxfId="15"/>
+    <tableColumn id="7" name="Time" dataDxfId="14"/>
+    <tableColumn id="9" name="Time Finished" dataDxfId="1"/>
+    <tableColumn id="8" name="Vessel Type" dataDxfId="13"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table1" displayName="Table1" ref="A1:H84" headerRowCount="1" totalsRowShown="0" headerRowDxfId="13" tableBorderDxfId="12">
-  <autoFilter ref="A1:H84"/>
-  <tableColumns count="8">
-    <tableColumn id="1" name="No." dataDxfId="11"/>
-    <tableColumn id="2" name="Vessel" dataDxfId="10"/>
-    <tableColumn id="3" name="Service" dataDxfId="9"/>
-    <tableColumn id="4" name="Control Number" dataDxfId="8"/>
-    <tableColumn id="5" name="Voyage Number" dataDxfId="7"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table1" displayName="Table1" ref="A1:I84" headerRowCount="1" totalsRowShown="0" headerRowDxfId="12" tableBorderDxfId="11">
+  <autoFilter ref="A1:I84"/>
+  <tableColumns count="9">
+    <tableColumn id="1" name="No." dataDxfId="10"/>
+    <tableColumn id="2" name="Vessel" dataDxfId="9"/>
+    <tableColumn id="3" name="Service" dataDxfId="8"/>
+    <tableColumn id="4" name="Control Number" dataDxfId="7"/>
+    <tableColumn id="5" name="Voyage Number" dataDxfId="6"/>
     <tableColumn id="6" name="Date" dataDxfId="5"/>
-    <tableColumn id="8" name="Time" dataDxfId="6"/>
-    <tableColumn id="9" name="Vessel Type" dataDxfId="4"/>
+    <tableColumn id="8" name="Time" dataDxfId="4"/>
+    <tableColumn id="7" name="Time Finished" dataDxfId="2"/>
+    <tableColumn id="9" name="Vessel Type" dataDxfId="3"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1622,7 +1706,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I74"/>
+  <dimension ref="A1:J74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9.85546875" customWidth="1" min="1" max="1"/>
@@ -1633,6 +1717,7 @@
     <col width="20.7109375" customWidth="1" min="6" max="6"/>
     <col width="18.85546875" customWidth="1" min="7" max="7"/>
     <col width="21" customWidth="1" min="8" max="8"/>
+    <col width="25.85546875" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1" thickBot="1">
@@ -1673,10 +1758,15 @@
       </c>
       <c r="H1" s="37" t="inlineStr">
         <is>
+          <t>Time Finished</t>
+        </is>
+      </c>
+      <c r="I1" s="37" t="inlineStr">
+        <is>
           <t>Vessel Type</t>
         </is>
       </c>
-      <c r="I1" s="12" t="n"/>
+      <c r="J1" s="12" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="13" t="n">
@@ -1707,6 +1797,7 @@
       </c>
       <c r="G2" s="35" t="n"/>
       <c r="H2" s="35" t="n"/>
+      <c r="I2" s="35" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="14" t="n">
@@ -1737,6 +1828,7 @@
       </c>
       <c r="G3" s="16" t="n"/>
       <c r="H3" s="16" t="n"/>
+      <c r="I3" s="16" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="14" t="n">
@@ -1765,6 +1857,7 @@
       </c>
       <c r="G4" s="16" t="n"/>
       <c r="H4" s="16" t="n"/>
+      <c r="I4" s="16" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="14" t="n">
@@ -1795,6 +1888,7 @@
       </c>
       <c r="G5" s="16" t="n"/>
       <c r="H5" s="16" t="n"/>
+      <c r="I5" s="16" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="14" t="n">
@@ -1825,6 +1919,7 @@
       </c>
       <c r="G6" s="16" t="n"/>
       <c r="H6" s="16" t="n"/>
+      <c r="I6" s="16" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="14" t="n">
@@ -1855,6 +1950,7 @@
       </c>
       <c r="G7" s="16" t="n"/>
       <c r="H7" s="16" t="n"/>
+      <c r="I7" s="16" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="14" t="n">
@@ -1885,6 +1981,7 @@
       </c>
       <c r="G8" s="16" t="n"/>
       <c r="H8" s="16" t="n"/>
+      <c r="I8" s="16" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="14" t="n">
@@ -1915,6 +2012,7 @@
       </c>
       <c r="G9" s="16" t="n"/>
       <c r="H9" s="16" t="n"/>
+      <c r="I9" s="16" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="14" t="n">
@@ -1945,6 +2043,7 @@
       </c>
       <c r="G10" s="16" t="n"/>
       <c r="H10" s="16" t="n"/>
+      <c r="I10" s="16" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="14" t="n">
@@ -1975,6 +2074,7 @@
       </c>
       <c r="G11" s="16" t="n"/>
       <c r="H11" s="16" t="n"/>
+      <c r="I11" s="16" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="14" t="n">
@@ -2005,6 +2105,7 @@
       </c>
       <c r="G12" s="16" t="n"/>
       <c r="H12" s="16" t="n"/>
+      <c r="I12" s="16" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="14" t="n">
@@ -2035,6 +2136,7 @@
       </c>
       <c r="G13" s="16" t="n"/>
       <c r="H13" s="16" t="n"/>
+      <c r="I13" s="16" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="14" t="n">
@@ -2065,6 +2167,7 @@
       </c>
       <c r="G14" s="16" t="n"/>
       <c r="H14" s="16" t="n"/>
+      <c r="I14" s="16" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="14" t="n">
@@ -2095,6 +2198,7 @@
       </c>
       <c r="G15" s="16" t="n"/>
       <c r="H15" s="16" t="n"/>
+      <c r="I15" s="16" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="14" t="n">
@@ -2125,6 +2229,7 @@
       </c>
       <c r="G16" s="16" t="n"/>
       <c r="H16" s="16" t="n"/>
+      <c r="I16" s="16" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="14" t="n">
@@ -2155,6 +2260,7 @@
       </c>
       <c r="G17" s="16" t="n"/>
       <c r="H17" s="16" t="n"/>
+      <c r="I17" s="16" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="14" t="n">
@@ -2185,6 +2291,7 @@
       </c>
       <c r="G18" s="16" t="n"/>
       <c r="H18" s="16" t="n"/>
+      <c r="I18" s="16" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="14" t="n">
@@ -2215,6 +2322,7 @@
       </c>
       <c r="G19" s="16" t="n"/>
       <c r="H19" s="16" t="n"/>
+      <c r="I19" s="16" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="14" t="n">
@@ -2245,6 +2353,7 @@
       </c>
       <c r="G20" s="16" t="n"/>
       <c r="H20" s="16" t="n"/>
+      <c r="I20" s="16" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="14" t="n">
@@ -2275,6 +2384,7 @@
       </c>
       <c r="G21" s="16" t="n"/>
       <c r="H21" s="16" t="n"/>
+      <c r="I21" s="16" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="14" t="n">
@@ -2305,6 +2415,7 @@
       </c>
       <c r="G22" s="16" t="n"/>
       <c r="H22" s="16" t="n"/>
+      <c r="I22" s="16" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="14" t="n">
@@ -2335,6 +2446,7 @@
       </c>
       <c r="G23" s="16" t="n"/>
       <c r="H23" s="16" t="n"/>
+      <c r="I23" s="16" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="14" t="n">
@@ -2365,6 +2477,7 @@
       </c>
       <c r="G24" s="16" t="n"/>
       <c r="H24" s="16" t="n"/>
+      <c r="I24" s="16" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="14" t="n">
@@ -2395,6 +2508,7 @@
       </c>
       <c r="G25" s="16" t="n"/>
       <c r="H25" s="16" t="n"/>
+      <c r="I25" s="16" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="14" t="n">
@@ -2425,6 +2539,7 @@
       </c>
       <c r="G26" s="16" t="n"/>
       <c r="H26" s="16" t="n"/>
+      <c r="I26" s="16" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="14" t="n">
@@ -2455,6 +2570,7 @@
       </c>
       <c r="G27" s="16" t="n"/>
       <c r="H27" s="16" t="n"/>
+      <c r="I27" s="16" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="14" t="n">
@@ -2485,6 +2601,7 @@
       </c>
       <c r="G28" s="16" t="n"/>
       <c r="H28" s="16" t="n"/>
+      <c r="I28" s="16" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="14" t="n">
@@ -2515,6 +2632,7 @@
       </c>
       <c r="G29" s="16" t="n"/>
       <c r="H29" s="16" t="n"/>
+      <c r="I29" s="16" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="14" t="n">
@@ -2545,6 +2663,7 @@
       </c>
       <c r="G30" s="16" t="n"/>
       <c r="H30" s="16" t="n"/>
+      <c r="I30" s="16" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="14" t="n">
@@ -2575,6 +2694,7 @@
       </c>
       <c r="G31" s="16" t="n"/>
       <c r="H31" s="16" t="n"/>
+      <c r="I31" s="16" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="14" t="n">
@@ -2605,6 +2725,7 @@
       </c>
       <c r="G32" s="16" t="n"/>
       <c r="H32" s="16" t="n"/>
+      <c r="I32" s="16" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="14" t="n">
@@ -2635,6 +2756,7 @@
       </c>
       <c r="G33" s="16" t="n"/>
       <c r="H33" s="16" t="n"/>
+      <c r="I33" s="16" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="14" t="n">
@@ -2665,6 +2787,7 @@
       </c>
       <c r="G34" s="16" t="n"/>
       <c r="H34" s="16" t="n"/>
+      <c r="I34" s="16" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="14" t="n">
@@ -2695,6 +2818,7 @@
       </c>
       <c r="G35" s="16" t="n"/>
       <c r="H35" s="16" t="n"/>
+      <c r="I35" s="16" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="14" t="n">
@@ -2725,6 +2849,7 @@
       </c>
       <c r="G36" s="16" t="n"/>
       <c r="H36" s="16" t="n"/>
+      <c r="I36" s="16" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="14" t="n">
@@ -2755,6 +2880,7 @@
       </c>
       <c r="G37" s="16" t="n"/>
       <c r="H37" s="16" t="n"/>
+      <c r="I37" s="16" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="14" t="n">
@@ -2785,6 +2911,7 @@
       </c>
       <c r="G38" s="16" t="n"/>
       <c r="H38" s="16" t="n"/>
+      <c r="I38" s="16" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="14" t="n">
@@ -2815,6 +2942,7 @@
       </c>
       <c r="G39" s="16" t="n"/>
       <c r="H39" s="16" t="n"/>
+      <c r="I39" s="16" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="14" t="n">
@@ -2845,6 +2973,7 @@
       </c>
       <c r="G40" s="16" t="n"/>
       <c r="H40" s="16" t="n"/>
+      <c r="I40" s="16" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="14" t="n">
@@ -2875,6 +3004,7 @@
       </c>
       <c r="G41" s="16" t="n"/>
       <c r="H41" s="16" t="n"/>
+      <c r="I41" s="16" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="14" t="n">
@@ -2905,6 +3035,7 @@
       </c>
       <c r="G42" s="16" t="n"/>
       <c r="H42" s="16" t="n"/>
+      <c r="I42" s="16" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="14" t="n">
@@ -2935,6 +3066,7 @@
       </c>
       <c r="G43" s="16" t="n"/>
       <c r="H43" s="16" t="n"/>
+      <c r="I43" s="16" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="14" t="n">
@@ -2965,6 +3097,7 @@
       </c>
       <c r="G44" s="16" t="n"/>
       <c r="H44" s="16" t="n"/>
+      <c r="I44" s="16" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="14" t="n">
@@ -2995,6 +3128,7 @@
       </c>
       <c r="G45" s="16" t="n"/>
       <c r="H45" s="16" t="n"/>
+      <c r="I45" s="16" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="14" t="n">
@@ -3025,6 +3159,7 @@
       </c>
       <c r="G46" s="16" t="n"/>
       <c r="H46" s="16" t="n"/>
+      <c r="I46" s="16" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="14" t="n">
@@ -3055,6 +3190,7 @@
       </c>
       <c r="G47" s="16" t="n"/>
       <c r="H47" s="16" t="n"/>
+      <c r="I47" s="16" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="14" t="n">
@@ -3085,6 +3221,7 @@
       </c>
       <c r="G48" s="16" t="n"/>
       <c r="H48" s="16" t="n"/>
+      <c r="I48" s="16" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="14" t="n">
@@ -3115,6 +3252,7 @@
       </c>
       <c r="G49" s="16" t="n"/>
       <c r="H49" s="16" t="n"/>
+      <c r="I49" s="16" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="14" t="n">
@@ -3145,6 +3283,7 @@
       </c>
       <c r="G50" s="16" t="n"/>
       <c r="H50" s="16" t="n"/>
+      <c r="I50" s="16" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="14" t="n">
@@ -3175,6 +3314,7 @@
       </c>
       <c r="G51" s="16" t="n"/>
       <c r="H51" s="16" t="n"/>
+      <c r="I51" s="16" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="14" t="n">
@@ -3205,6 +3345,7 @@
       </c>
       <c r="G52" s="16" t="n"/>
       <c r="H52" s="16" t="n"/>
+      <c r="I52" s="16" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="14" t="n">
@@ -3235,6 +3376,7 @@
       </c>
       <c r="G53" s="16" t="n"/>
       <c r="H53" s="16" t="n"/>
+      <c r="I53" s="16" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="14" t="n">
@@ -3265,6 +3407,7 @@
       </c>
       <c r="G54" s="16" t="n"/>
       <c r="H54" s="16" t="n"/>
+      <c r="I54" s="16" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="14" t="n">
@@ -3295,6 +3438,7 @@
       </c>
       <c r="G55" s="16" t="n"/>
       <c r="H55" s="16" t="n"/>
+      <c r="I55" s="16" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="14" t="n">
@@ -3325,6 +3469,7 @@
       </c>
       <c r="G56" s="16" t="n"/>
       <c r="H56" s="16" t="n"/>
+      <c r="I56" s="16" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="14" t="n">
@@ -3355,6 +3500,7 @@
       </c>
       <c r="G57" s="16" t="n"/>
       <c r="H57" s="16" t="n"/>
+      <c r="I57" s="16" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="14" t="n">
@@ -3385,6 +3531,7 @@
       </c>
       <c r="G58" s="16" t="n"/>
       <c r="H58" s="16" t="n"/>
+      <c r="I58" s="16" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="14" t="n">
@@ -3415,6 +3562,7 @@
       </c>
       <c r="G59" s="16" t="n"/>
       <c r="H59" s="16" t="n"/>
+      <c r="I59" s="16" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="14" t="n">
@@ -3445,6 +3593,7 @@
       </c>
       <c r="G60" s="16" t="n"/>
       <c r="H60" s="16" t="n"/>
+      <c r="I60" s="16" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="14" t="n">
@@ -3475,6 +3624,7 @@
       </c>
       <c r="G61" s="16" t="n"/>
       <c r="H61" s="16" t="n"/>
+      <c r="I61" s="16" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="14" t="n">
@@ -3505,6 +3655,7 @@
       </c>
       <c r="G62" s="16" t="n"/>
       <c r="H62" s="16" t="n"/>
+      <c r="I62" s="16" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="14" t="n">
@@ -3535,6 +3686,7 @@
       </c>
       <c r="G63" s="16" t="n"/>
       <c r="H63" s="16" t="n"/>
+      <c r="I63" s="16" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="14" t="n">
@@ -3565,6 +3717,7 @@
       </c>
       <c r="G64" s="16" t="n"/>
       <c r="H64" s="16" t="n"/>
+      <c r="I64" s="16" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="14" t="n">
@@ -3595,6 +3748,7 @@
       </c>
       <c r="G65" s="16" t="n"/>
       <c r="H65" s="16" t="n"/>
+      <c r="I65" s="16" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="14" t="n">
@@ -3625,6 +3779,7 @@
       </c>
       <c r="G66" s="16" t="n"/>
       <c r="H66" s="16" t="n"/>
+      <c r="I66" s="16" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="14" t="n">
@@ -3655,6 +3810,7 @@
       </c>
       <c r="G67" s="16" t="n"/>
       <c r="H67" s="16" t="n"/>
+      <c r="I67" s="16" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="14" t="n">
@@ -3685,6 +3841,7 @@
       </c>
       <c r="G68" s="16" t="n"/>
       <c r="H68" s="16" t="n"/>
+      <c r="I68" s="16" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="14" t="n">
@@ -3715,6 +3872,7 @@
       </c>
       <c r="G69" s="16" t="n"/>
       <c r="H69" s="16" t="n"/>
+      <c r="I69" s="16" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="14" t="n">
@@ -3745,6 +3903,7 @@
       </c>
       <c r="G70" s="16" t="n"/>
       <c r="H70" s="16" t="n"/>
+      <c r="I70" s="16" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="14" t="n">
@@ -3775,6 +3934,7 @@
       </c>
       <c r="G71" s="16" t="n"/>
       <c r="H71" s="16" t="n"/>
+      <c r="I71" s="16" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="14" t="n">
@@ -3805,6 +3965,7 @@
       </c>
       <c r="G72" s="16" t="n"/>
       <c r="H72" s="16" t="n"/>
+      <c r="I72" s="16" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="14" t="n">
@@ -3835,6 +3996,7 @@
       </c>
       <c r="G73" s="16" t="n"/>
       <c r="H73" s="16" t="n"/>
+      <c r="I73" s="16" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="20" t="n">
@@ -3865,6 +4027,7 @@
       </c>
       <c r="G74" s="23" t="n"/>
       <c r="H74" s="23" t="n"/>
+      <c r="I74" s="23" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3880,7 +4043,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H148"/>
+  <dimension ref="A1:I148"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15.85546875" customWidth="1" min="1" max="1"/>
@@ -3891,6 +4054,8 @@
     <col width="16.5703125" bestFit="1" customWidth="1" min="6" max="6"/>
     <col width="20.28515625" customWidth="1" min="7" max="7"/>
     <col width="21.140625" customWidth="1" min="8" max="8"/>
+    <col width="21.28515625" customWidth="1" min="9" max="9"/>
+    <col width="19" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1" thickBot="1">
@@ -3931,6 +4096,11 @@
       </c>
       <c r="H1" s="18" t="inlineStr">
         <is>
+          <t>Time Finished</t>
+        </is>
+      </c>
+      <c r="I1" s="18" t="inlineStr">
+        <is>
           <t>Vessel Type</t>
         </is>
       </c>
@@ -3964,6 +4134,7 @@
       </c>
       <c r="G2" s="36" t="n"/>
       <c r="H2" s="36" t="n"/>
+      <c r="I2" s="36" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="25" t="n">
@@ -3994,6 +4165,7 @@
       </c>
       <c r="G3" s="27" t="n"/>
       <c r="H3" s="27" t="n"/>
+      <c r="I3" s="27" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="25" t="n">
@@ -4024,6 +4196,7 @@
       </c>
       <c r="G4" s="27" t="n"/>
       <c r="H4" s="27" t="n"/>
+      <c r="I4" s="27" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="25" t="n">
@@ -4054,6 +4227,7 @@
       </c>
       <c r="G5" s="27" t="n"/>
       <c r="H5" s="27" t="n"/>
+      <c r="I5" s="27" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="25" t="n">
@@ -4084,6 +4258,7 @@
       </c>
       <c r="G6" s="27" t="n"/>
       <c r="H6" s="27" t="n"/>
+      <c r="I6" s="27" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="25" t="n">
@@ -4114,6 +4289,7 @@
       </c>
       <c r="G7" s="27" t="n"/>
       <c r="H7" s="27" t="n"/>
+      <c r="I7" s="27" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="25" t="n">
@@ -4144,6 +4320,7 @@
       </c>
       <c r="G8" s="27" t="n"/>
       <c r="H8" s="27" t="n"/>
+      <c r="I8" s="27" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="25" t="n">
@@ -4174,6 +4351,7 @@
       </c>
       <c r="G9" s="27" t="n"/>
       <c r="H9" s="27" t="n"/>
+      <c r="I9" s="27" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="25" t="n">
@@ -4204,6 +4382,7 @@
       </c>
       <c r="G10" s="27" t="n"/>
       <c r="H10" s="27" t="n"/>
+      <c r="I10" s="27" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="25" t="n">
@@ -4234,6 +4413,7 @@
       </c>
       <c r="G11" s="27" t="n"/>
       <c r="H11" s="27" t="n"/>
+      <c r="I11" s="27" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="25" t="n">
@@ -4264,6 +4444,7 @@
       </c>
       <c r="G12" s="27" t="n"/>
       <c r="H12" s="27" t="n"/>
+      <c r="I12" s="27" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="25" t="n">
@@ -4294,6 +4475,7 @@
       </c>
       <c r="G13" s="27" t="n"/>
       <c r="H13" s="27" t="n"/>
+      <c r="I13" s="27" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="25" t="n">
@@ -4324,6 +4506,7 @@
       </c>
       <c r="G14" s="27" t="n"/>
       <c r="H14" s="27" t="n"/>
+      <c r="I14" s="27" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="25" t="n">
@@ -4354,6 +4537,7 @@
       </c>
       <c r="G15" s="27" t="n"/>
       <c r="H15" s="27" t="n"/>
+      <c r="I15" s="27" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="25" t="n">
@@ -4384,6 +4568,7 @@
       </c>
       <c r="G16" s="27" t="n"/>
       <c r="H16" s="27" t="n"/>
+      <c r="I16" s="27" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="25" t="n">
@@ -4414,6 +4599,7 @@
       </c>
       <c r="G17" s="27" t="n"/>
       <c r="H17" s="27" t="n"/>
+      <c r="I17" s="27" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="25" t="n">
@@ -4444,6 +4630,7 @@
       </c>
       <c r="G18" s="27" t="n"/>
       <c r="H18" s="27" t="n"/>
+      <c r="I18" s="27" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="25" t="n">
@@ -4474,6 +4661,7 @@
       </c>
       <c r="G19" s="27" t="n"/>
       <c r="H19" s="27" t="n"/>
+      <c r="I19" s="27" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="25" t="n">
@@ -4504,6 +4692,7 @@
       </c>
       <c r="G20" s="27" t="n"/>
       <c r="H20" s="27" t="n"/>
+      <c r="I20" s="27" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="25" t="n">
@@ -4534,6 +4723,7 @@
       </c>
       <c r="G21" s="27" t="n"/>
       <c r="H21" s="27" t="n"/>
+      <c r="I21" s="27" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="25" t="n">
@@ -4564,6 +4754,7 @@
       </c>
       <c r="G22" s="27" t="n"/>
       <c r="H22" s="27" t="n"/>
+      <c r="I22" s="27" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="25" t="n">
@@ -4594,6 +4785,7 @@
       </c>
       <c r="G23" s="27" t="n"/>
       <c r="H23" s="27" t="n"/>
+      <c r="I23" s="27" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="25" t="n">
@@ -4624,6 +4816,7 @@
       </c>
       <c r="G24" s="27" t="n"/>
       <c r="H24" s="27" t="n"/>
+      <c r="I24" s="27" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="25" t="n">
@@ -4654,6 +4847,7 @@
       </c>
       <c r="G25" s="27" t="n"/>
       <c r="H25" s="27" t="n"/>
+      <c r="I25" s="27" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="25" t="n">
@@ -4684,6 +4878,7 @@
       </c>
       <c r="G26" s="27" t="n"/>
       <c r="H26" s="27" t="n"/>
+      <c r="I26" s="27" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="25" t="n">
@@ -4714,6 +4909,7 @@
       </c>
       <c r="G27" s="27" t="n"/>
       <c r="H27" s="27" t="n"/>
+      <c r="I27" s="27" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="25" t="n">
@@ -4744,6 +4940,7 @@
       </c>
       <c r="G28" s="27" t="n"/>
       <c r="H28" s="27" t="n"/>
+      <c r="I28" s="27" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="25" t="n">
@@ -4774,6 +4971,7 @@
       </c>
       <c r="G29" s="27" t="n"/>
       <c r="H29" s="27" t="n"/>
+      <c r="I29" s="27" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="25" t="n">
@@ -4804,6 +5002,7 @@
       </c>
       <c r="G30" s="27" t="n"/>
       <c r="H30" s="27" t="n"/>
+      <c r="I30" s="27" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="25" t="n">
@@ -4834,6 +5033,7 @@
       </c>
       <c r="G31" s="27" t="n"/>
       <c r="H31" s="27" t="n"/>
+      <c r="I31" s="27" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="25" t="n">
@@ -4864,6 +5064,7 @@
       </c>
       <c r="G32" s="27" t="n"/>
       <c r="H32" s="27" t="n"/>
+      <c r="I32" s="27" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="25" t="n">
@@ -4894,6 +5095,7 @@
       </c>
       <c r="G33" s="27" t="n"/>
       <c r="H33" s="27" t="n"/>
+      <c r="I33" s="27" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="25" t="n">
@@ -4924,6 +5126,7 @@
       </c>
       <c r="G34" s="27" t="n"/>
       <c r="H34" s="27" t="n"/>
+      <c r="I34" s="27" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="25" t="n">
@@ -4954,6 +5157,7 @@
       </c>
       <c r="G35" s="27" t="n"/>
       <c r="H35" s="27" t="n"/>
+      <c r="I35" s="27" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="25" t="n">
@@ -4984,6 +5188,7 @@
       </c>
       <c r="G36" s="27" t="n"/>
       <c r="H36" s="27" t="n"/>
+      <c r="I36" s="27" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="25" t="n">
@@ -5014,6 +5219,7 @@
       </c>
       <c r="G37" s="27" t="n"/>
       <c r="H37" s="27" t="n"/>
+      <c r="I37" s="27" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="25" t="n">
@@ -5044,6 +5250,7 @@
       </c>
       <c r="G38" s="27" t="n"/>
       <c r="H38" s="27" t="n"/>
+      <c r="I38" s="27" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="25" t="n">
@@ -5074,6 +5281,7 @@
       </c>
       <c r="G39" s="27" t="n"/>
       <c r="H39" s="27" t="n"/>
+      <c r="I39" s="27" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="25" t="n">
@@ -5104,6 +5312,7 @@
       </c>
       <c r="G40" s="27" t="n"/>
       <c r="H40" s="27" t="n"/>
+      <c r="I40" s="27" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="25" t="n">
@@ -5134,6 +5343,7 @@
       </c>
       <c r="G41" s="27" t="n"/>
       <c r="H41" s="27" t="n"/>
+      <c r="I41" s="27" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="25" t="n">
@@ -5164,6 +5374,7 @@
       </c>
       <c r="G42" s="27" t="n"/>
       <c r="H42" s="27" t="n"/>
+      <c r="I42" s="27" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="25" t="n">
@@ -5194,6 +5405,7 @@
       </c>
       <c r="G43" s="27" t="n"/>
       <c r="H43" s="27" t="n"/>
+      <c r="I43" s="27" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="25" t="n">
@@ -5224,6 +5436,7 @@
       </c>
       <c r="G44" s="27" t="n"/>
       <c r="H44" s="27" t="n"/>
+      <c r="I44" s="27" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="25" t="n">
@@ -5254,6 +5467,7 @@
       </c>
       <c r="G45" s="27" t="n"/>
       <c r="H45" s="27" t="n"/>
+      <c r="I45" s="27" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="25" t="n">
@@ -5284,6 +5498,7 @@
       </c>
       <c r="G46" s="27" t="n"/>
       <c r="H46" s="27" t="n"/>
+      <c r="I46" s="27" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="25" t="n">
@@ -5314,6 +5529,7 @@
       </c>
       <c r="G47" s="27" t="n"/>
       <c r="H47" s="27" t="n"/>
+      <c r="I47" s="27" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="25" t="n">
@@ -5344,6 +5560,7 @@
       </c>
       <c r="G48" s="27" t="n"/>
       <c r="H48" s="27" t="n"/>
+      <c r="I48" s="27" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="25" t="n">
@@ -5374,6 +5591,7 @@
       </c>
       <c r="G49" s="27" t="n"/>
       <c r="H49" s="27" t="n"/>
+      <c r="I49" s="27" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="25" t="n">
@@ -5404,6 +5622,7 @@
       </c>
       <c r="G50" s="27" t="n"/>
       <c r="H50" s="27" t="n"/>
+      <c r="I50" s="27" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="25" t="n">
@@ -5434,6 +5653,7 @@
       </c>
       <c r="G51" s="27" t="n"/>
       <c r="H51" s="27" t="n"/>
+      <c r="I51" s="27" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="25" t="n">
@@ -5464,6 +5684,7 @@
       </c>
       <c r="G52" s="27" t="n"/>
       <c r="H52" s="27" t="n"/>
+      <c r="I52" s="27" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="25" t="n">
@@ -5494,6 +5715,7 @@
       </c>
       <c r="G53" s="27" t="n"/>
       <c r="H53" s="27" t="n"/>
+      <c r="I53" s="27" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="25" t="n">
@@ -5524,6 +5746,7 @@
       </c>
       <c r="G54" s="27" t="n"/>
       <c r="H54" s="27" t="n"/>
+      <c r="I54" s="27" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="25" t="n">
@@ -5554,6 +5777,7 @@
       </c>
       <c r="G55" s="27" t="n"/>
       <c r="H55" s="27" t="n"/>
+      <c r="I55" s="27" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="25" t="n">
@@ -5584,6 +5808,7 @@
       </c>
       <c r="G56" s="27" t="n"/>
       <c r="H56" s="27" t="n"/>
+      <c r="I56" s="27" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="25" t="n">
@@ -5614,6 +5839,7 @@
       </c>
       <c r="G57" s="27" t="n"/>
       <c r="H57" s="27" t="n"/>
+      <c r="I57" s="27" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="25" t="n">
@@ -5644,6 +5870,7 @@
       </c>
       <c r="G58" s="27" t="n"/>
       <c r="H58" s="27" t="n"/>
+      <c r="I58" s="27" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="25" t="n">
@@ -5674,6 +5901,7 @@
       </c>
       <c r="G59" s="27" t="n"/>
       <c r="H59" s="27" t="n"/>
+      <c r="I59" s="27" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="25" t="n">
@@ -5704,6 +5932,7 @@
       </c>
       <c r="G60" s="27" t="n"/>
       <c r="H60" s="27" t="n"/>
+      <c r="I60" s="27" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="25" t="n">
@@ -5734,6 +5963,7 @@
       </c>
       <c r="G61" s="27" t="n"/>
       <c r="H61" s="27" t="n"/>
+      <c r="I61" s="27" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="25" t="n">
@@ -5764,6 +5994,7 @@
       </c>
       <c r="G62" s="27" t="n"/>
       <c r="H62" s="27" t="n"/>
+      <c r="I62" s="27" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="25" t="n">
@@ -5794,6 +6025,7 @@
       </c>
       <c r="G63" s="27" t="n"/>
       <c r="H63" s="27" t="n"/>
+      <c r="I63" s="27" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="25" t="n">
@@ -5824,6 +6056,7 @@
       </c>
       <c r="G64" s="27" t="n"/>
       <c r="H64" s="27" t="n"/>
+      <c r="I64" s="27" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="25" t="n">
@@ -5854,6 +6087,7 @@
       </c>
       <c r="G65" s="27" t="n"/>
       <c r="H65" s="27" t="n"/>
+      <c r="I65" s="27" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="25" t="n">
@@ -5884,6 +6118,7 @@
       </c>
       <c r="G66" s="27" t="n"/>
       <c r="H66" s="27" t="n"/>
+      <c r="I66" s="27" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="25" t="n">
@@ -5914,6 +6149,7 @@
       </c>
       <c r="G67" s="27" t="n"/>
       <c r="H67" s="27" t="n"/>
+      <c r="I67" s="27" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="25" t="n">
@@ -5944,6 +6180,7 @@
       </c>
       <c r="G68" s="27" t="n"/>
       <c r="H68" s="27" t="n"/>
+      <c r="I68" s="27" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="25" t="n">
@@ -5974,6 +6211,7 @@
       </c>
       <c r="G69" s="27" t="n"/>
       <c r="H69" s="27" t="n"/>
+      <c r="I69" s="27" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="25" t="n">
@@ -6004,6 +6242,7 @@
       </c>
       <c r="G70" s="27" t="n"/>
       <c r="H70" s="27" t="n"/>
+      <c r="I70" s="27" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="25" t="n">
@@ -6034,6 +6273,7 @@
       </c>
       <c r="G71" s="27" t="n"/>
       <c r="H71" s="27" t="n"/>
+      <c r="I71" s="27" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="25" t="n">
@@ -6064,6 +6304,7 @@
       </c>
       <c r="G72" s="27" t="n"/>
       <c r="H72" s="27" t="n"/>
+      <c r="I72" s="27" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="25" t="n">
@@ -6094,6 +6335,7 @@
       </c>
       <c r="G73" s="27" t="n"/>
       <c r="H73" s="27" t="n"/>
+      <c r="I73" s="27" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="25" t="n">
@@ -6124,6 +6366,7 @@
       </c>
       <c r="G74" s="27" t="n"/>
       <c r="H74" s="27" t="n"/>
+      <c r="I74" s="27" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="25" t="n">
@@ -6154,6 +6397,7 @@
       </c>
       <c r="G75" s="27" t="n"/>
       <c r="H75" s="27" t="n"/>
+      <c r="I75" s="27" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="25" t="n">
@@ -6184,6 +6428,7 @@
       </c>
       <c r="G76" s="27" t="n"/>
       <c r="H76" s="27" t="n"/>
+      <c r="I76" s="27" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="25" t="n">
@@ -6214,6 +6459,7 @@
       </c>
       <c r="G77" s="27" t="n"/>
       <c r="H77" s="27" t="n"/>
+      <c r="I77" s="27" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="25" t="n">
@@ -6244,6 +6490,7 @@
       </c>
       <c r="G78" s="27" t="n"/>
       <c r="H78" s="27" t="n"/>
+      <c r="I78" s="27" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="25" t="n">
@@ -6274,6 +6521,7 @@
       </c>
       <c r="G79" s="27" t="n"/>
       <c r="H79" s="27" t="n"/>
+      <c r="I79" s="27" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="25" t="n">
@@ -6304,6 +6552,7 @@
       </c>
       <c r="G80" s="27" t="n"/>
       <c r="H80" s="27" t="n"/>
+      <c r="I80" s="27" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="25" t="n">
@@ -6334,6 +6583,7 @@
       </c>
       <c r="G81" s="27" t="n"/>
       <c r="H81" s="27" t="n"/>
+      <c r="I81" s="27" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="25" t="n">
@@ -6364,6 +6614,7 @@
       </c>
       <c r="G82" s="27" t="n"/>
       <c r="H82" s="27" t="n"/>
+      <c r="I82" s="27" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="25" t="n">
@@ -6394,6 +6645,7 @@
       </c>
       <c r="G83" s="27" t="n"/>
       <c r="H83" s="27" t="n"/>
+      <c r="I83" s="27" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="25" t="n">
@@ -6424,6 +6676,7 @@
       </c>
       <c r="G84" s="27" t="n"/>
       <c r="H84" s="27" t="n"/>
+      <c r="I84" s="27" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="25" t="n">
@@ -6454,6 +6707,7 @@
       </c>
       <c r="G85" s="27" t="n"/>
       <c r="H85" s="27" t="n"/>
+      <c r="I85" s="27" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="25" t="n">
@@ -6484,6 +6738,7 @@
       </c>
       <c r="G86" s="27" t="n"/>
       <c r="H86" s="27" t="n"/>
+      <c r="I86" s="27" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="25" t="n">
@@ -6514,6 +6769,7 @@
       </c>
       <c r="G87" s="27" t="n"/>
       <c r="H87" s="27" t="n"/>
+      <c r="I87" s="27" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="25" t="n">
@@ -6544,6 +6800,7 @@
       </c>
       <c r="G88" s="27" t="n"/>
       <c r="H88" s="27" t="n"/>
+      <c r="I88" s="27" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="25" t="n">
@@ -6574,6 +6831,7 @@
       </c>
       <c r="G89" s="27" t="n"/>
       <c r="H89" s="27" t="n"/>
+      <c r="I89" s="27" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="25" t="n">
@@ -6604,6 +6862,7 @@
       </c>
       <c r="G90" s="27" t="n"/>
       <c r="H90" s="27" t="n"/>
+      <c r="I90" s="27" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="25" t="n">
@@ -6634,6 +6893,7 @@
       </c>
       <c r="G91" s="27" t="n"/>
       <c r="H91" s="27" t="n"/>
+      <c r="I91" s="27" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="25" t="n">
@@ -6664,6 +6924,7 @@
       </c>
       <c r="G92" s="27" t="n"/>
       <c r="H92" s="27" t="n"/>
+      <c r="I92" s="27" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="25" t="n">
@@ -6694,6 +6955,7 @@
       </c>
       <c r="G93" s="27" t="n"/>
       <c r="H93" s="27" t="n"/>
+      <c r="I93" s="27" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="25" t="n">
@@ -6724,6 +6986,7 @@
       </c>
       <c r="G94" s="27" t="n"/>
       <c r="H94" s="27" t="n"/>
+      <c r="I94" s="27" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="25" t="n">
@@ -6754,6 +7017,7 @@
       </c>
       <c r="G95" s="27" t="n"/>
       <c r="H95" s="27" t="n"/>
+      <c r="I95" s="27" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="25" t="n">
@@ -6784,6 +7048,7 @@
       </c>
       <c r="G96" s="27" t="n"/>
       <c r="H96" s="27" t="n"/>
+      <c r="I96" s="27" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="25" t="n">
@@ -6814,6 +7079,7 @@
       </c>
       <c r="G97" s="27" t="n"/>
       <c r="H97" s="27" t="n"/>
+      <c r="I97" s="27" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="25" t="n">
@@ -6844,6 +7110,7 @@
       </c>
       <c r="G98" s="27" t="n"/>
       <c r="H98" s="27" t="n"/>
+      <c r="I98" s="27" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="25" t="n">
@@ -6874,6 +7141,7 @@
       </c>
       <c r="G99" s="27" t="n"/>
       <c r="H99" s="27" t="n"/>
+      <c r="I99" s="27" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="25" t="n">
@@ -6904,6 +7172,7 @@
       </c>
       <c r="G100" s="27" t="n"/>
       <c r="H100" s="27" t="n"/>
+      <c r="I100" s="27" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="25" t="n">
@@ -6934,6 +7203,7 @@
       </c>
       <c r="G101" s="27" t="n"/>
       <c r="H101" s="27" t="n"/>
+      <c r="I101" s="27" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="25" t="n">
@@ -6964,6 +7234,7 @@
       </c>
       <c r="G102" s="27" t="n"/>
       <c r="H102" s="27" t="n"/>
+      <c r="I102" s="27" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="25" t="n">
@@ -6994,6 +7265,7 @@
       </c>
       <c r="G103" s="27" t="n"/>
       <c r="H103" s="27" t="n"/>
+      <c r="I103" s="27" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="25" t="n">
@@ -7024,6 +7296,7 @@
       </c>
       <c r="G104" s="27" t="n"/>
       <c r="H104" s="27" t="n"/>
+      <c r="I104" s="27" t="n"/>
     </row>
     <row r="105">
       <c r="A105" s="25" t="n">
@@ -7054,6 +7327,7 @@
       </c>
       <c r="G105" s="27" t="n"/>
       <c r="H105" s="27" t="n"/>
+      <c r="I105" s="27" t="n"/>
     </row>
     <row r="106">
       <c r="A106" s="25" t="n">
@@ -7084,6 +7358,7 @@
       </c>
       <c r="G106" s="27" t="n"/>
       <c r="H106" s="27" t="n"/>
+      <c r="I106" s="27" t="n"/>
     </row>
     <row r="107">
       <c r="A107" s="25" t="n">
@@ -7114,6 +7389,7 @@
       </c>
       <c r="G107" s="27" t="n"/>
       <c r="H107" s="27" t="n"/>
+      <c r="I107" s="27" t="n"/>
     </row>
     <row r="108">
       <c r="A108" s="25" t="n">
@@ -7144,6 +7420,7 @@
       </c>
       <c r="G108" s="27" t="n"/>
       <c r="H108" s="27" t="n"/>
+      <c r="I108" s="27" t="n"/>
     </row>
     <row r="109">
       <c r="A109" s="25" t="n">
@@ -7174,6 +7451,7 @@
       </c>
       <c r="G109" s="27" t="n"/>
       <c r="H109" s="27" t="n"/>
+      <c r="I109" s="27" t="n"/>
     </row>
     <row r="110">
       <c r="A110" s="25" t="n">
@@ -7204,6 +7482,7 @@
       </c>
       <c r="G110" s="27" t="n"/>
       <c r="H110" s="27" t="n"/>
+      <c r="I110" s="27" t="n"/>
     </row>
     <row r="111">
       <c r="A111" s="25" t="n">
@@ -7234,6 +7513,7 @@
       </c>
       <c r="G111" s="27" t="n"/>
       <c r="H111" s="27" t="n"/>
+      <c r="I111" s="27" t="n"/>
     </row>
     <row r="112">
       <c r="A112" s="25" t="n">
@@ -7264,6 +7544,7 @@
       </c>
       <c r="G112" s="27" t="n"/>
       <c r="H112" s="27" t="n"/>
+      <c r="I112" s="27" t="n"/>
     </row>
     <row r="113">
       <c r="A113" s="25" t="n">
@@ -7294,6 +7575,7 @@
       </c>
       <c r="G113" s="27" t="n"/>
       <c r="H113" s="27" t="n"/>
+      <c r="I113" s="27" t="n"/>
     </row>
     <row r="114">
       <c r="A114" s="25" t="n">
@@ -7324,6 +7606,7 @@
       </c>
       <c r="G114" s="27" t="n"/>
       <c r="H114" s="27" t="n"/>
+      <c r="I114" s="27" t="n"/>
     </row>
     <row r="115">
       <c r="A115" s="25" t="n">
@@ -7354,6 +7637,7 @@
       </c>
       <c r="G115" s="27" t="n"/>
       <c r="H115" s="27" t="n"/>
+      <c r="I115" s="27" t="n"/>
     </row>
     <row r="116">
       <c r="A116" s="25" t="n">
@@ -7384,6 +7668,7 @@
       </c>
       <c r="G116" s="27" t="n"/>
       <c r="H116" s="27" t="n"/>
+      <c r="I116" s="27" t="n"/>
     </row>
     <row r="117">
       <c r="A117" s="25" t="n">
@@ -7414,6 +7699,7 @@
       </c>
       <c r="G117" s="27" t="n"/>
       <c r="H117" s="27" t="n"/>
+      <c r="I117" s="27" t="n"/>
     </row>
     <row r="118">
       <c r="A118" s="25" t="n">
@@ -7444,6 +7730,7 @@
       </c>
       <c r="G118" s="27" t="n"/>
       <c r="H118" s="27" t="n"/>
+      <c r="I118" s="27" t="n"/>
     </row>
     <row r="119">
       <c r="A119" s="25" t="n">
@@ -7474,6 +7761,7 @@
       </c>
       <c r="G119" s="27" t="n"/>
       <c r="H119" s="27" t="n"/>
+      <c r="I119" s="27" t="n"/>
     </row>
     <row r="120">
       <c r="A120" s="25" t="n">
@@ -7504,6 +7792,7 @@
       </c>
       <c r="G120" s="27" t="n"/>
       <c r="H120" s="27" t="n"/>
+      <c r="I120" s="27" t="n"/>
     </row>
     <row r="121">
       <c r="A121" s="25" t="n">
@@ -7534,6 +7823,7 @@
       </c>
       <c r="G121" s="27" t="n"/>
       <c r="H121" s="27" t="n"/>
+      <c r="I121" s="27" t="n"/>
     </row>
     <row r="122">
       <c r="A122" s="25" t="n">
@@ -7564,6 +7854,7 @@
       </c>
       <c r="G122" s="27" t="n"/>
       <c r="H122" s="27" t="n"/>
+      <c r="I122" s="27" t="n"/>
     </row>
     <row r="123">
       <c r="A123" s="25" t="n">
@@ -7594,6 +7885,7 @@
       </c>
       <c r="G123" s="27" t="n"/>
       <c r="H123" s="27" t="n"/>
+      <c r="I123" s="27" t="n"/>
     </row>
     <row r="124">
       <c r="A124" s="25" t="n">
@@ -7624,6 +7916,7 @@
       </c>
       <c r="G124" s="27" t="n"/>
       <c r="H124" s="27" t="n"/>
+      <c r="I124" s="27" t="n"/>
     </row>
     <row r="125">
       <c r="A125" s="25" t="n">
@@ -7654,6 +7947,7 @@
       </c>
       <c r="G125" s="27" t="n"/>
       <c r="H125" s="27" t="n"/>
+      <c r="I125" s="27" t="n"/>
     </row>
     <row r="126">
       <c r="A126" s="25" t="n">
@@ -7684,6 +7978,7 @@
       </c>
       <c r="G126" s="27" t="n"/>
       <c r="H126" s="27" t="n"/>
+      <c r="I126" s="27" t="n"/>
     </row>
     <row r="127">
       <c r="A127" s="25" t="n">
@@ -7714,6 +8009,7 @@
       </c>
       <c r="G127" s="27" t="n"/>
       <c r="H127" s="27" t="n"/>
+      <c r="I127" s="27" t="n"/>
     </row>
     <row r="128">
       <c r="A128" s="25" t="n">
@@ -7744,6 +8040,7 @@
       </c>
       <c r="G128" s="27" t="n"/>
       <c r="H128" s="27" t="n"/>
+      <c r="I128" s="27" t="n"/>
     </row>
     <row r="129">
       <c r="A129" s="25" t="n">
@@ -7774,6 +8071,7 @@
       </c>
       <c r="G129" s="27" t="n"/>
       <c r="H129" s="27" t="n"/>
+      <c r="I129" s="27" t="n"/>
     </row>
     <row r="130">
       <c r="A130" s="25" t="n">
@@ -7804,6 +8102,7 @@
       </c>
       <c r="G130" s="27" t="n"/>
       <c r="H130" s="27" t="n"/>
+      <c r="I130" s="27" t="n"/>
     </row>
     <row r="131">
       <c r="A131" s="25" t="n">
@@ -7834,6 +8133,7 @@
       </c>
       <c r="G131" s="27" t="n"/>
       <c r="H131" s="27" t="n"/>
+      <c r="I131" s="27" t="n"/>
     </row>
     <row r="132">
       <c r="A132" s="25" t="n">
@@ -7864,6 +8164,7 @@
       </c>
       <c r="G132" s="27" t="n"/>
       <c r="H132" s="27" t="n"/>
+      <c r="I132" s="27" t="n"/>
     </row>
     <row r="133">
       <c r="A133" s="25" t="n">
@@ -7894,6 +8195,7 @@
       </c>
       <c r="G133" s="27" t="n"/>
       <c r="H133" s="27" t="n"/>
+      <c r="I133" s="27" t="n"/>
     </row>
     <row r="134">
       <c r="A134" s="25" t="n">
@@ -7924,6 +8226,7 @@
       </c>
       <c r="G134" s="27" t="n"/>
       <c r="H134" s="27" t="n"/>
+      <c r="I134" s="27" t="n"/>
     </row>
     <row r="135">
       <c r="A135" s="25" t="n">
@@ -7954,6 +8257,7 @@
       </c>
       <c r="G135" s="27" t="n"/>
       <c r="H135" s="27" t="n"/>
+      <c r="I135" s="27" t="n"/>
     </row>
     <row r="136">
       <c r="A136" s="25" t="n">
@@ -7984,6 +8288,7 @@
       </c>
       <c r="G136" s="27" t="n"/>
       <c r="H136" s="27" t="n"/>
+      <c r="I136" s="27" t="n"/>
     </row>
     <row r="137">
       <c r="A137" s="25" t="n">
@@ -8014,6 +8319,7 @@
       </c>
       <c r="G137" s="27" t="n"/>
       <c r="H137" s="27" t="n"/>
+      <c r="I137" s="27" t="n"/>
     </row>
     <row r="138">
       <c r="A138" s="25" t="n">
@@ -8044,6 +8350,7 @@
       </c>
       <c r="G138" s="27" t="n"/>
       <c r="H138" s="27" t="n"/>
+      <c r="I138" s="27" t="n"/>
     </row>
     <row r="139">
       <c r="A139" s="25" t="n">
@@ -8074,6 +8381,7 @@
       </c>
       <c r="G139" s="27" t="n"/>
       <c r="H139" s="27" t="n"/>
+      <c r="I139" s="27" t="n"/>
     </row>
     <row r="140">
       <c r="A140" s="25" t="n">
@@ -8104,6 +8412,7 @@
       </c>
       <c r="G140" s="27" t="n"/>
       <c r="H140" s="27" t="n"/>
+      <c r="I140" s="27" t="n"/>
     </row>
     <row r="141">
       <c r="A141" s="25" t="n">
@@ -8134,6 +8443,7 @@
       </c>
       <c r="G141" s="27" t="n"/>
       <c r="H141" s="27" t="n"/>
+      <c r="I141" s="27" t="n"/>
     </row>
     <row r="142">
       <c r="A142" s="25" t="n">
@@ -8164,6 +8474,7 @@
       </c>
       <c r="G142" s="27" t="n"/>
       <c r="H142" s="27" t="n"/>
+      <c r="I142" s="27" t="n"/>
     </row>
     <row r="143">
       <c r="A143" s="25" t="n">
@@ -8194,6 +8505,7 @@
       </c>
       <c r="G143" s="27" t="n"/>
       <c r="H143" s="27" t="n"/>
+      <c r="I143" s="27" t="n"/>
     </row>
     <row r="144">
       <c r="A144" s="25" t="n">
@@ -8224,6 +8536,7 @@
       </c>
       <c r="G144" s="27" t="n"/>
       <c r="H144" s="27" t="n"/>
+      <c r="I144" s="27" t="n"/>
     </row>
     <row r="145">
       <c r="A145" s="25" t="n">
@@ -8254,6 +8567,7 @@
       </c>
       <c r="G145" s="27" t="n"/>
       <c r="H145" s="27" t="n"/>
+      <c r="I145" s="27" t="n"/>
     </row>
     <row r="146">
       <c r="A146" s="25" t="n">
@@ -8284,6 +8598,7 @@
       </c>
       <c r="G146" s="27" t="n"/>
       <c r="H146" s="27" t="n"/>
+      <c r="I146" s="27" t="n"/>
     </row>
     <row r="147">
       <c r="A147" s="25" t="n">
@@ -8314,6 +8629,7 @@
       </c>
       <c r="G147" s="27" t="n"/>
       <c r="H147" s="27" t="n"/>
+      <c r="I147" s="27" t="n"/>
     </row>
     <row r="148">
       <c r="A148" s="28" t="n">
@@ -8344,6 +8660,7 @@
       </c>
       <c r="G148" s="31" t="n"/>
       <c r="H148" s="31" t="n"/>
+      <c r="I148" s="31" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -8359,7 +8676,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H89"/>
+  <dimension ref="A1:I91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15.85546875" customWidth="1" min="1" max="1"/>
@@ -8369,6 +8686,7 @@
     <col width="25.85546875" customWidth="1" min="5" max="6"/>
     <col width="16.5703125" bestFit="1" customWidth="1" min="7" max="7"/>
     <col width="26" customWidth="1" min="8" max="8"/>
+    <col width="21.28515625" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -8409,6 +8727,11 @@
       </c>
       <c r="H1" s="19" t="inlineStr">
         <is>
+          <t>Time Finished</t>
+        </is>
+      </c>
+      <c r="I1" s="19" t="inlineStr">
+        <is>
           <t>Vessel Type</t>
         </is>
       </c>
@@ -8442,6 +8765,7 @@
       </c>
       <c r="G2" s="16" t="n"/>
       <c r="H2" s="16" t="n"/>
+      <c r="I2" s="16" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="14" t="n">
@@ -8472,6 +8796,7 @@
       </c>
       <c r="G3" s="16" t="n"/>
       <c r="H3" s="16" t="n"/>
+      <c r="I3" s="16" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="14" t="n">
@@ -8502,6 +8827,7 @@
       </c>
       <c r="G4" s="16" t="n"/>
       <c r="H4" s="16" t="n"/>
+      <c r="I4" s="16" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="14" t="n">
@@ -8532,6 +8858,7 @@
       </c>
       <c r="G5" s="16" t="n"/>
       <c r="H5" s="16" t="n"/>
+      <c r="I5" s="16" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="14" t="n">
@@ -8562,6 +8889,7 @@
       </c>
       <c r="G6" s="16" t="n"/>
       <c r="H6" s="16" t="n"/>
+      <c r="I6" s="16" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="14" t="n">
@@ -8592,6 +8920,7 @@
       </c>
       <c r="G7" s="16" t="n"/>
       <c r="H7" s="16" t="n"/>
+      <c r="I7" s="16" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="14" t="n">
@@ -8624,6 +8953,7 @@
       </c>
       <c r="G8" s="16" t="n"/>
       <c r="H8" s="16" t="n"/>
+      <c r="I8" s="16" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="14" t="n">
@@ -8654,6 +8984,7 @@
       </c>
       <c r="G9" s="16" t="n"/>
       <c r="H9" s="16" t="n"/>
+      <c r="I9" s="16" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="14" t="n">
@@ -8684,6 +9015,7 @@
       </c>
       <c r="G10" s="16" t="n"/>
       <c r="H10" s="16" t="n"/>
+      <c r="I10" s="16" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="14" t="n">
@@ -8714,6 +9046,7 @@
       </c>
       <c r="G11" s="16" t="n"/>
       <c r="H11" s="16" t="n"/>
+      <c r="I11" s="16" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="14" t="n">
@@ -8744,6 +9077,7 @@
       </c>
       <c r="G12" s="16" t="n"/>
       <c r="H12" s="16" t="n"/>
+      <c r="I12" s="16" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="14" t="n">
@@ -8774,6 +9108,7 @@
       </c>
       <c r="G13" s="16" t="n"/>
       <c r="H13" s="16" t="n"/>
+      <c r="I13" s="16" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="14" t="n">
@@ -8804,6 +9139,7 @@
       </c>
       <c r="G14" s="16" t="n"/>
       <c r="H14" s="16" t="n"/>
+      <c r="I14" s="16" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="14" t="n">
@@ -8834,6 +9170,7 @@
       </c>
       <c r="G15" s="16" t="n"/>
       <c r="H15" s="16" t="n"/>
+      <c r="I15" s="16" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="14" t="n">
@@ -8864,6 +9201,7 @@
       </c>
       <c r="G16" s="16" t="n"/>
       <c r="H16" s="16" t="n"/>
+      <c r="I16" s="16" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="14" t="n">
@@ -8894,6 +9232,7 @@
       </c>
       <c r="G17" s="16" t="n"/>
       <c r="H17" s="16" t="n"/>
+      <c r="I17" s="16" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="14" t="n">
@@ -8924,6 +9263,7 @@
       </c>
       <c r="G18" s="16" t="n"/>
       <c r="H18" s="16" t="n"/>
+      <c r="I18" s="16" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="14" t="n">
@@ -8954,6 +9294,7 @@
       </c>
       <c r="G19" s="16" t="n"/>
       <c r="H19" s="16" t="n"/>
+      <c r="I19" s="16" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="14" t="n">
@@ -8984,6 +9325,7 @@
       </c>
       <c r="G20" s="16" t="n"/>
       <c r="H20" s="16" t="n"/>
+      <c r="I20" s="16" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="14" t="n">
@@ -9014,6 +9356,7 @@
       </c>
       <c r="G21" s="16" t="n"/>
       <c r="H21" s="16" t="n"/>
+      <c r="I21" s="16" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="14" t="n">
@@ -9044,6 +9387,7 @@
       </c>
       <c r="G22" s="16" t="n"/>
       <c r="H22" s="16" t="n"/>
+      <c r="I22" s="16" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="14" t="n">
@@ -9074,6 +9418,7 @@
       </c>
       <c r="G23" s="16" t="n"/>
       <c r="H23" s="16" t="n"/>
+      <c r="I23" s="16" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="14" t="n">
@@ -9104,6 +9449,7 @@
       </c>
       <c r="G24" s="16" t="n"/>
       <c r="H24" s="16" t="n"/>
+      <c r="I24" s="16" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="14" t="n">
@@ -9134,6 +9480,7 @@
       </c>
       <c r="G25" s="16" t="n"/>
       <c r="H25" s="16" t="n"/>
+      <c r="I25" s="16" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="14" t="n">
@@ -9164,6 +9511,7 @@
       </c>
       <c r="G26" s="16" t="n"/>
       <c r="H26" s="16" t="n"/>
+      <c r="I26" s="16" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="14" t="n">
@@ -9194,6 +9542,7 @@
       </c>
       <c r="G27" s="16" t="n"/>
       <c r="H27" s="16" t="n"/>
+      <c r="I27" s="16" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="14" t="n">
@@ -9224,6 +9573,7 @@
       </c>
       <c r="G28" s="16" t="n"/>
       <c r="H28" s="16" t="n"/>
+      <c r="I28" s="16" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="14" t="n">
@@ -9254,6 +9604,7 @@
       </c>
       <c r="G29" s="16" t="n"/>
       <c r="H29" s="16" t="n"/>
+      <c r="I29" s="16" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="14" t="n">
@@ -9284,6 +9635,7 @@
       </c>
       <c r="G30" s="16" t="n"/>
       <c r="H30" s="16" t="n"/>
+      <c r="I30" s="16" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="14" t="n">
@@ -9314,6 +9666,7 @@
       </c>
       <c r="G31" s="16" t="n"/>
       <c r="H31" s="16" t="n"/>
+      <c r="I31" s="16" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="14" t="n">
@@ -9344,6 +9697,7 @@
       </c>
       <c r="G32" s="16" t="n"/>
       <c r="H32" s="16" t="n"/>
+      <c r="I32" s="16" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="14" t="n">
@@ -9374,6 +9728,7 @@
       </c>
       <c r="G33" s="16" t="n"/>
       <c r="H33" s="16" t="n"/>
+      <c r="I33" s="16" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="14" t="n">
@@ -9404,6 +9759,7 @@
       </c>
       <c r="G34" s="16" t="n"/>
       <c r="H34" s="16" t="n"/>
+      <c r="I34" s="16" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="14" t="n">
@@ -9434,6 +9790,7 @@
       </c>
       <c r="G35" s="16" t="n"/>
       <c r="H35" s="16" t="n"/>
+      <c r="I35" s="16" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="14" t="n">
@@ -9464,6 +9821,7 @@
       </c>
       <c r="G36" s="16" t="n"/>
       <c r="H36" s="16" t="n"/>
+      <c r="I36" s="16" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="14" t="n">
@@ -9494,6 +9852,7 @@
       </c>
       <c r="G37" s="16" t="n"/>
       <c r="H37" s="16" t="n"/>
+      <c r="I37" s="16" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="14" t="n">
@@ -9524,6 +9883,7 @@
       </c>
       <c r="G38" s="16" t="n"/>
       <c r="H38" s="16" t="n"/>
+      <c r="I38" s="16" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="14" t="n">
@@ -9554,6 +9914,7 @@
       </c>
       <c r="G39" s="16" t="n"/>
       <c r="H39" s="16" t="n"/>
+      <c r="I39" s="16" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="14" t="n">
@@ -9584,6 +9945,7 @@
       </c>
       <c r="G40" s="16" t="n"/>
       <c r="H40" s="16" t="n"/>
+      <c r="I40" s="16" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="14" t="n">
@@ -9614,6 +9976,7 @@
       </c>
       <c r="G41" s="16" t="n"/>
       <c r="H41" s="16" t="n"/>
+      <c r="I41" s="16" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="14" t="n">
@@ -9644,6 +10007,7 @@
       </c>
       <c r="G42" s="16" t="n"/>
       <c r="H42" s="16" t="n"/>
+      <c r="I42" s="16" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="14" t="n">
@@ -9674,6 +10038,7 @@
       </c>
       <c r="G43" s="16" t="n"/>
       <c r="H43" s="16" t="n"/>
+      <c r="I43" s="16" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="14" t="n">
@@ -9704,6 +10069,7 @@
       </c>
       <c r="G44" s="16" t="n"/>
       <c r="H44" s="16" t="n"/>
+      <c r="I44" s="16" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="14" t="n">
@@ -9734,6 +10100,7 @@
       </c>
       <c r="G45" s="16" t="n"/>
       <c r="H45" s="16" t="n"/>
+      <c r="I45" s="16" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="14" t="n">
@@ -9764,6 +10131,7 @@
       </c>
       <c r="G46" s="16" t="n"/>
       <c r="H46" s="16" t="n"/>
+      <c r="I46" s="16" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="14" t="n">
@@ -9794,6 +10162,7 @@
       </c>
       <c r="G47" s="16" t="n"/>
       <c r="H47" s="16" t="n"/>
+      <c r="I47" s="16" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="14" t="n">
@@ -9824,6 +10193,7 @@
       </c>
       <c r="G48" s="16" t="n"/>
       <c r="H48" s="16" t="n"/>
+      <c r="I48" s="16" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="14" t="n">
@@ -9854,6 +10224,7 @@
       </c>
       <c r="G49" s="16" t="n"/>
       <c r="H49" s="16" t="n"/>
+      <c r="I49" s="16" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="14" t="n">
@@ -9884,6 +10255,7 @@
       </c>
       <c r="G50" s="16" t="n"/>
       <c r="H50" s="16" t="n"/>
+      <c r="I50" s="16" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="14" t="n">
@@ -9914,6 +10286,7 @@
       </c>
       <c r="G51" s="16" t="n"/>
       <c r="H51" s="16" t="n"/>
+      <c r="I51" s="16" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="14" t="n">
@@ -9944,6 +10317,7 @@
       </c>
       <c r="G52" s="16" t="n"/>
       <c r="H52" s="16" t="n"/>
+      <c r="I52" s="16" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="14" t="n">
@@ -9974,6 +10348,7 @@
       </c>
       <c r="G53" s="16" t="n"/>
       <c r="H53" s="16" t="n"/>
+      <c r="I53" s="16" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="14" t="n">
@@ -10004,6 +10379,7 @@
       </c>
       <c r="G54" s="16" t="n"/>
       <c r="H54" s="16" t="n"/>
+      <c r="I54" s="16" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="14" t="n">
@@ -10034,6 +10410,7 @@
       </c>
       <c r="G55" s="16" t="n"/>
       <c r="H55" s="16" t="n"/>
+      <c r="I55" s="16" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="14" t="n">
@@ -10064,6 +10441,7 @@
       </c>
       <c r="G56" s="16" t="n"/>
       <c r="H56" s="16" t="n"/>
+      <c r="I56" s="16" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="14" t="n">
@@ -10094,6 +10472,7 @@
       </c>
       <c r="G57" s="16" t="n"/>
       <c r="H57" s="16" t="n"/>
+      <c r="I57" s="16" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="14" t="n">
@@ -10124,6 +10503,7 @@
       </c>
       <c r="G58" s="16" t="n"/>
       <c r="H58" s="16" t="n"/>
+      <c r="I58" s="16" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="14" t="n">
@@ -10154,6 +10534,7 @@
       </c>
       <c r="G59" s="16" t="n"/>
       <c r="H59" s="16" t="n"/>
+      <c r="I59" s="16" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="14" t="n">
@@ -10184,6 +10565,7 @@
       </c>
       <c r="G60" s="16" t="n"/>
       <c r="H60" s="16" t="n"/>
+      <c r="I60" s="16" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="14" t="n">
@@ -10214,6 +10596,7 @@
       </c>
       <c r="G61" s="16" t="n"/>
       <c r="H61" s="16" t="n"/>
+      <c r="I61" s="16" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="14" t="n">
@@ -10244,6 +10627,7 @@
       </c>
       <c r="G62" s="16" t="n"/>
       <c r="H62" s="16" t="n"/>
+      <c r="I62" s="16" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="14" t="n">
@@ -10274,6 +10658,7 @@
       </c>
       <c r="G63" s="16" t="n"/>
       <c r="H63" s="16" t="n"/>
+      <c r="I63" s="16" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="14" t="n">
@@ -10304,6 +10689,7 @@
       </c>
       <c r="G64" s="16" t="n"/>
       <c r="H64" s="16" t="n"/>
+      <c r="I64" s="16" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="14" t="n">
@@ -10334,6 +10720,7 @@
       </c>
       <c r="G65" s="16" t="n"/>
       <c r="H65" s="16" t="n"/>
+      <c r="I65" s="16" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="14" t="n">
@@ -10364,6 +10751,7 @@
       </c>
       <c r="G66" s="16" t="n"/>
       <c r="H66" s="16" t="n"/>
+      <c r="I66" s="16" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="14" t="n">
@@ -10394,6 +10782,7 @@
       </c>
       <c r="G67" s="16" t="n"/>
       <c r="H67" s="16" t="n"/>
+      <c r="I67" s="16" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="14" t="n">
@@ -10424,6 +10813,7 @@
       </c>
       <c r="G68" s="16" t="n"/>
       <c r="H68" s="16" t="n"/>
+      <c r="I68" s="16" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="14" t="n">
@@ -10454,6 +10844,7 @@
       </c>
       <c r="G69" s="16" t="n"/>
       <c r="H69" s="16" t="n"/>
+      <c r="I69" s="16" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="14" t="n">
@@ -10484,6 +10875,7 @@
       </c>
       <c r="G70" s="16" t="n"/>
       <c r="H70" s="16" t="n"/>
+      <c r="I70" s="16" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="14" t="n">
@@ -10514,6 +10906,7 @@
       </c>
       <c r="G71" s="16" t="n"/>
       <c r="H71" s="16" t="n"/>
+      <c r="I71" s="16" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="14" t="n">
@@ -10544,6 +10937,7 @@
       </c>
       <c r="G72" s="16" t="n"/>
       <c r="H72" s="16" t="n"/>
+      <c r="I72" s="16" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="14" t="n">
@@ -10574,6 +10968,7 @@
       </c>
       <c r="G73" s="16" t="n"/>
       <c r="H73" s="16" t="n"/>
+      <c r="I73" s="16" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="14" t="n">
@@ -10604,6 +10999,7 @@
       </c>
       <c r="G74" s="16" t="n"/>
       <c r="H74" s="16" t="n"/>
+      <c r="I74" s="16" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="14" t="n">
@@ -10634,6 +11030,7 @@
       </c>
       <c r="G75" s="16" t="n"/>
       <c r="H75" s="16" t="n"/>
+      <c r="I75" s="16" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="14" t="n">
@@ -10664,6 +11061,7 @@
       </c>
       <c r="G76" s="16" t="n"/>
       <c r="H76" s="16" t="n"/>
+      <c r="I76" s="16" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="14" t="n">
@@ -10694,6 +11092,7 @@
       </c>
       <c r="G77" s="16" t="n"/>
       <c r="H77" s="16" t="n"/>
+      <c r="I77" s="16" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="14" t="n">
@@ -10724,6 +11123,7 @@
       </c>
       <c r="G78" s="16" t="n"/>
       <c r="H78" s="16" t="n"/>
+      <c r="I78" s="16" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="14" t="n">
@@ -10754,6 +11154,7 @@
       </c>
       <c r="G79" s="16" t="n"/>
       <c r="H79" s="16" t="n"/>
+      <c r="I79" s="16" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="14" t="n">
@@ -10784,6 +11185,7 @@
       </c>
       <c r="G80" s="16" t="n"/>
       <c r="H80" s="16" t="n"/>
+      <c r="I80" s="16" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="14" t="n">
@@ -10814,6 +11216,7 @@
       </c>
       <c r="G81" s="16" t="n"/>
       <c r="H81" s="16" t="n"/>
+      <c r="I81" s="16" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="14" t="n">
@@ -10844,6 +11247,7 @@
       </c>
       <c r="G82" s="16" t="n"/>
       <c r="H82" s="16" t="n"/>
+      <c r="I82" s="16" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="14" t="n">
@@ -10874,6 +11278,7 @@
       </c>
       <c r="G83" s="16" t="n"/>
       <c r="H83" s="16" t="n"/>
+      <c r="I83" s="16" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="20" t="n">
@@ -10904,6 +11309,7 @@
       </c>
       <c r="G84" s="23" t="n"/>
       <c r="H84" s="23" t="n"/>
+      <c r="I84" s="23" t="n"/>
     </row>
     <row r="85">
       <c r="A85" t="n">
@@ -10939,7 +11345,7 @@
           <t>04:09</t>
         </is>
       </c>
-      <c r="H85" t="inlineStr">
+      <c r="I85" t="inlineStr">
         <is>
           <t>Local</t>
         </is>
@@ -10979,7 +11385,7 @@
           <t>08:02</t>
         </is>
       </c>
-      <c r="H86" t="inlineStr">
+      <c r="I86" t="inlineStr">
         <is>
           <t>Foreign</t>
         </is>
@@ -11019,7 +11425,7 @@
           <t>08:02</t>
         </is>
       </c>
-      <c r="H87" t="inlineStr">
+      <c r="I87" t="inlineStr">
         <is>
           <t>Local</t>
         </is>
@@ -11059,7 +11465,7 @@
           <t>10:31</t>
         </is>
       </c>
-      <c r="H88" t="inlineStr">
+      <c r="I88" t="inlineStr">
         <is>
           <t>Local</t>
         </is>
@@ -11099,7 +11505,97 @@
           <t>10:36</t>
         </is>
       </c>
-      <c r="H89" t="inlineStr">
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="n">
+        <v>89</v>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>testtt</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>W/ MOORING BUOY</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>testtt</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>testtt</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>2025-11-02</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>10:07</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>10:12</t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="n">
+        <v>90</v>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>testtt1</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>W/ MOORING BUOY</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>testtt1</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>testtt1</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>2025-11-03</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>10:59 AM</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>11:03 AM</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
         <is>
           <t>Local</t>
         </is>

</xml_diff>